<commit_message>
docs: resequence worksheets and update demo timetable
</commit_message>
<xml_diff>
--- a/module_schedule.xlsx
+++ b/module_schedule.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2" conformance="strict">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30431"/>
   <workbookPr dateCompatibility="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://portdotacdotuk-my.sharepoint.com/personal/mani_ghahremani_port_ac_uk/Documents/_Docs/Work Docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EA3DF98B-3883-435B-9CF2-82C977038B12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E5038DCD-2C1E-4B4A-9BD1-504799618AFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="18960" xr2:uid="{268B58E5-37B1-4943-A657-E8A6B83DFA17}"/>
   </bookViews>
@@ -46,9 +46,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="42" uniqueCount="39">
-  <si>
-    <t>Week ending Monday</t>
+<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="40" uniqueCount="37">
+  <si>
+    <t>Week beginning Monday</t>
   </si>
   <si>
     <t>Week ending Friday</t>
@@ -60,24 +60,18 @@
     <t>Lecture</t>
   </si>
   <si>
-    <t>Demo</t>
-  </si>
-  <si>
-    <t>Worksheet 0</t>
-  </si>
-  <si>
-    <t>Lecture 0</t>
+    <t>Assessments</t>
+  </si>
+  <si>
+    <t>Worksheet 1</t>
+  </si>
+  <si>
+    <t>Lecture 1</t>
   </si>
   <si>
     <t>Demo 1</t>
   </si>
   <si>
-    <t>Worksheet 1</t>
-  </si>
-  <si>
-    <t>Lecture 1</t>
-  </si>
-  <si>
     <t>Worksheet 2</t>
   </si>
   <si>
@@ -108,7 +102,7 @@
     <t>Demo 3</t>
   </si>
   <si>
-    <t>Reading Week</t>
+    <t>Break</t>
   </si>
   <si>
     <t>Worksheet 6</t>
@@ -169,9 +163,6 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="m/d/yyyy"/>
-  </numFmts>
   <fonts count="8">
     <font>
       <sz val="11"/>
@@ -264,7 +255,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="37">
+  <borders count="36">
     <border>
       <start/>
       <end/>
@@ -524,17 +515,6 @@
         <color rgb="FF000000"/>
       </end>
       <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <start style="medium">
-        <color rgb="FF000000"/>
-      </start>
-      <end style="thin">
-        <color rgb="FF000000"/>
-      </end>
-      <top/>
       <bottom style="medium">
         <color rgb="FF000000"/>
       </bottom>
@@ -712,7 +692,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -720,173 +700,170 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -915,13 +892,13 @@
   <xdr:twoCellAnchor editAs="absolute">
     <xdr:from>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>247650</xdr:colOff>
+      <xdr:colOff>561975</xdr:colOff>
       <xdr:row>105</xdr:row>
       <xdr:rowOff>79375</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>692150</xdr:colOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>130175</xdr:colOff>
       <xdr:row>113</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
@@ -1013,13 +990,13 @@
   <xdr:twoCellAnchor editAs="absolute">
     <xdr:from>
       <xdr:col>21</xdr:col>
-      <xdr:colOff>904875</xdr:colOff>
+      <xdr:colOff>1219200</xdr:colOff>
       <xdr:row>105</xdr:row>
       <xdr:rowOff>79375</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>22</xdr:col>
-      <xdr:colOff>939800</xdr:colOff>
+      <xdr:colOff>1254125</xdr:colOff>
       <xdr:row>113</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
@@ -1110,14 +1087,14 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="absolute">
     <xdr:from>
-      <xdr:col>28</xdr:col>
-      <xdr:colOff>1247775</xdr:colOff>
+      <xdr:col>29</xdr:col>
+      <xdr:colOff>276225</xdr:colOff>
       <xdr:row>105</xdr:row>
       <xdr:rowOff>79375</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>29</xdr:col>
-      <xdr:colOff>1282700</xdr:colOff>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>311150</xdr:colOff>
       <xdr:row>113</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
@@ -1209,13 +1186,13 @@
   <xdr:twoCellAnchor editAs="absolute">
     <xdr:from>
       <xdr:col>31</xdr:col>
-      <xdr:colOff>504825</xdr:colOff>
+      <xdr:colOff>819150</xdr:colOff>
       <xdr:row>105</xdr:row>
       <xdr:rowOff>79375</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>32</xdr:col>
-      <xdr:colOff>539750</xdr:colOff>
+      <xdr:colOff>854075</xdr:colOff>
       <xdr:row>113</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
@@ -1627,12 +1604,11 @@
   <sheetPr>
     <tabColor rgb="FF95B3D7"/>
   </sheetPr>
-  <dimension ref="A1:E936"/>
+  <dimension ref="A1:E935"/>
   <sheetFormatPr defaultColWidth="16.875" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="2" width="19.625" customWidth="1"/>
-    <col min="3" max="4" width="20.75" customWidth="1"/>
-    <col min="5" max="5" width="11.5" style="24" customWidth="1"/>
+    <col min="1" max="4" width="17.625" customWidth="1"/>
+    <col min="5" max="5" width="17.625" style="8" customWidth="1"/>
     <col min="6" max="20" width="11.5" customWidth="1"/>
     <col min="21" max="21" width="16.875" customWidth="1"/>
   </cols>
@@ -1650,16 +1626,16 @@
       <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="19" t="s">
+      <c r="E1" s="6" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="14.25">
       <c r="A2" s="3" t="d">
-        <v>2026-09-14</v>
+        <v>2026-09-21</v>
       </c>
       <c r="B2" s="4" t="d">
-        <v>2026-09-18</v>
+        <v>2026-09-25</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>5</v>
@@ -1667,16 +1643,16 @@
       <c r="D2" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="E2" s="20" t="s">
+      <c r="E2" s="38" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="14.25">
+    <row r="3" spans="1:5" ht="14.25" customHeight="1">
       <c r="A3" s="3" t="d">
-        <v>2026-09-21</v>
+        <v>2026-09-28</v>
       </c>
       <c r="B3" s="4" t="d">
-        <v>2026-09-25</v>
+        <v>2026-10-02</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>8</v>
@@ -1684,14 +1660,14 @@
       <c r="D3" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="21"/>
+      <c r="E3" s="39"/>
     </row>
     <row r="4" spans="1:5" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="d">
-        <v>2026-09-28</v>
+        <v>2026-10-05</v>
       </c>
       <c r="B4" s="4" t="d">
-        <v>2026-10-02</v>
+        <v>2026-10-09</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>10</v>
@@ -1699,31 +1675,31 @@
       <c r="D4" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E4" s="22"/>
+      <c r="E4" s="38" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="5" spans="1:5" ht="14.25" customHeight="1">
       <c r="A5" s="3" t="d">
-        <v>2026-10-05</v>
+        <v>2026-10-12</v>
       </c>
       <c r="B5" s="4" t="d">
-        <v>2026-10-09</v>
+        <v>2026-10-16</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E5" s="20" t="s">
         <v>14</v>
       </c>
+      <c r="E5" s="39"/>
     </row>
     <row r="6" spans="1:5" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="d">
-        <v>2026-10-12</v>
+        <v>2026-10-19</v>
       </c>
       <c r="B6" s="4" t="d">
-        <v>2026-10-16</v>
+        <v>2026-10-23</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>15</v>
@@ -1731,44 +1707,46 @@
       <c r="D6" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="E6" s="22"/>
-    </row>
-    <row r="7" spans="1:5" ht="14.25" customHeight="1">
+      <c r="E6" s="7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="14.25">
       <c r="A7" s="3" t="d">
-        <v>2026-10-19</v>
+        <v>2026-10-26</v>
       </c>
       <c r="B7" s="4" t="d">
-        <v>2026-10-23</v>
-      </c>
-      <c r="C7" s="5" t="s">
+        <v>2026-10-30</v>
+      </c>
+      <c r="C7" s="41" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" s="42"/>
+      <c r="E7" s="43"/>
+    </row>
+    <row r="8" spans="1:5" ht="15" customHeight="1">
+      <c r="A8" s="3" t="d">
+        <v>2026-11-02</v>
+      </c>
+      <c r="B8" s="4" t="d">
+        <v>2026-11-06</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E8" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="D7" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="E7" s="23" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="14.25">
-      <c r="A8" s="3" t="d">
-        <v>2026-10-26</v>
-      </c>
-      <c r="B8" s="4" t="d">
-        <v>2026-10-30</v>
-      </c>
-      <c r="C8" s="57" t="s">
-        <v>20</v>
-      </c>
-      <c r="D8" s="58"/>
-      <c r="E8" s="59"/>
-    </row>
-    <row r="9" spans="1:5" ht="15" customHeight="1">
+    </row>
+    <row r="9" spans="1:5" ht="14.25" customHeight="1">
       <c r="A9" s="3" t="d">
-        <v>2026-11-02</v>
+        <v>2026-11-09</v>
       </c>
       <c r="B9" s="4" t="d">
-        <v>2026-11-06</v>
+        <v>2026-11-13</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>21</v>
@@ -1776,33 +1754,31 @@
       <c r="D9" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="E9" s="23" t="s">
-        <v>19</v>
+      <c r="E9" s="38" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="14.25" customHeight="1">
       <c r="A10" s="3" t="d">
-        <v>2026-11-09</v>
+        <v>2026-11-16</v>
       </c>
       <c r="B10" s="4" t="d">
-        <v>2026-11-13</v>
+        <v>2026-11-20</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="E10" s="20" t="s">
         <v>25</v>
       </c>
+      <c r="E10" s="39"/>
     </row>
     <row r="11" spans="1:5" ht="14.25" customHeight="1">
       <c r="A11" s="3" t="d">
-        <v>2026-11-16</v>
+        <v>2026-11-23</v>
       </c>
       <c r="B11" s="4" t="d">
-        <v>2026-11-20</v>
+        <v>2026-11-27</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>26</v>
@@ -1810,277 +1786,263 @@
       <c r="D11" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="E11" s="22"/>
+      <c r="E11" s="38" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="12" spans="1:5" ht="14.25" customHeight="1">
       <c r="A12" s="3" t="d">
-        <v>2026-11-23</v>
+        <v>2026-11-30</v>
       </c>
       <c r="B12" s="4" t="d">
-        <v>2026-11-27</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="D12" s="5" t="s">
+        <v>2026-12-04</v>
+      </c>
+      <c r="C12" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="E12" s="20" t="s">
+      <c r="D12" s="10" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" ht="14.25" customHeight="1">
-      <c r="A13" s="3" t="d">
-        <v>2026-11-30</v>
-      </c>
-      <c r="B13" s="4" t="d">
-        <v>2026-12-04</v>
-      </c>
-      <c r="C13" s="55" t="s">
+      <c r="E12" s="40"/>
+    </row>
+    <row r="13" spans="1:5" ht="14.25">
+      <c r="A13" s="13" t="d">
+        <v>2026-12-07</v>
+      </c>
+      <c r="B13" s="11" t="d">
+        <v>2026-12-18</v>
+      </c>
+      <c r="C13" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="D13" s="55" t="s">
+      <c r="D13" s="18"/>
+      <c r="E13" s="19"/>
+    </row>
+    <row r="14" spans="1:5" ht="14.25">
+      <c r="A14" s="14"/>
+      <c r="B14" s="12"/>
+      <c r="C14" s="20"/>
+      <c r="D14" s="21"/>
+      <c r="E14" s="22"/>
+    </row>
+    <row r="15" spans="1:5" ht="14.25" customHeight="1">
+      <c r="A15" s="13" t="d">
+        <v>2026-12-21</v>
+      </c>
+      <c r="B15" s="11" t="d">
+        <v>2026-01-08</v>
+      </c>
+      <c r="C15" s="23" t="s">
         <v>32</v>
       </c>
-      <c r="E13" s="56"/>
-    </row>
-    <row r="14" spans="1:5" ht="14.25">
-      <c r="A14" s="6" t="d">
-        <v>2026-12-07</v>
-      </c>
-      <c r="B14" s="51" t="d">
-        <v>2026-12-18</v>
-      </c>
-      <c r="C14" s="25" t="s">
+      <c r="D15" s="24"/>
+      <c r="E15" s="25"/>
+    </row>
+    <row r="16" spans="1:5" ht="14.25" customHeight="1">
+      <c r="A16" s="15"/>
+      <c r="B16" s="16"/>
+      <c r="C16" s="26"/>
+      <c r="D16" s="27"/>
+      <c r="E16" s="28"/>
+    </row>
+    <row r="17" spans="1:5" ht="14.25" customHeight="1">
+      <c r="A17" s="14"/>
+      <c r="B17" s="12"/>
+      <c r="C17" s="29"/>
+      <c r="D17" s="30"/>
+      <c r="E17" s="31"/>
+    </row>
+    <row r="18" spans="1:5" ht="14.25">
+      <c r="A18" s="3" t="d">
+        <v>2027-01-11</v>
+      </c>
+      <c r="B18" s="9" t="d">
+        <v>2027-01-15</v>
+      </c>
+      <c r="C18" s="32" t="s">
         <v>33</v>
       </c>
-      <c r="D14" s="26"/>
-      <c r="E14" s="27"/>
-    </row>
-    <row r="15" spans="1:5" ht="14.25">
-      <c r="A15" s="8"/>
-      <c r="B15" s="52"/>
-      <c r="C15" s="28"/>
-      <c r="D15" s="10"/>
-      <c r="E15" s="29"/>
-    </row>
-    <row r="16" spans="1:5" ht="14.25" customHeight="1">
-      <c r="A16" s="6" t="d">
-        <v>2026-12-21</v>
-      </c>
-      <c r="B16" s="51" t="d">
-        <v>2026-01-08</v>
-      </c>
-      <c r="C16" s="30" t="s">
+      <c r="D18" s="33"/>
+      <c r="E18" s="34"/>
+    </row>
+    <row r="19" spans="1:5" ht="14.25">
+      <c r="A19" s="13" t="d">
+        <v>2027-01-18</v>
+      </c>
+      <c r="B19" s="11" t="d">
+        <v>2027-03-21</v>
+      </c>
+      <c r="C19" s="44" t="s">
         <v>34</v>
       </c>
-      <c r="D16" s="11"/>
-      <c r="E16" s="31"/>
-    </row>
-    <row r="17" spans="1:5" ht="14.25" customHeight="1">
-      <c r="A17" s="7"/>
-      <c r="B17" s="53"/>
-      <c r="C17" s="32"/>
-      <c r="D17" s="12"/>
-      <c r="E17" s="33"/>
-    </row>
-    <row r="18" spans="1:5" ht="14.25" customHeight="1">
-      <c r="A18" s="8"/>
-      <c r="B18" s="52"/>
-      <c r="C18" s="34"/>
-      <c r="D18" s="13"/>
-      <c r="E18" s="35"/>
-    </row>
-    <row r="19" spans="1:5" ht="14.25">
-      <c r="A19" s="3" t="d">
-        <v>2027-01-11</v>
-      </c>
-      <c r="B19" s="54" t="d">
-        <v>2027-01-15</v>
-      </c>
-      <c r="C19" s="36" t="s">
+      <c r="D19" s="45"/>
+      <c r="E19" s="46"/>
+    </row>
+    <row r="20" spans="1:5" ht="14.25" customHeight="1">
+      <c r="A20" s="15"/>
+      <c r="B20" s="16"/>
+      <c r="C20" s="47"/>
+      <c r="D20" s="48"/>
+      <c r="E20" s="49"/>
+    </row>
+    <row r="21" spans="1:5" ht="14.25" customHeight="1">
+      <c r="A21" s="15"/>
+      <c r="B21" s="16"/>
+      <c r="C21" s="47"/>
+      <c r="D21" s="48"/>
+      <c r="E21" s="49"/>
+    </row>
+    <row r="22" spans="1:5" ht="14.25" customHeight="1">
+      <c r="A22" s="15"/>
+      <c r="B22" s="16"/>
+      <c r="C22" s="47"/>
+      <c r="D22" s="48"/>
+      <c r="E22" s="49"/>
+    </row>
+    <row r="23" spans="1:5" ht="14.25" customHeight="1">
+      <c r="A23" s="15"/>
+      <c r="B23" s="16"/>
+      <c r="C23" s="47"/>
+      <c r="D23" s="48"/>
+      <c r="E23" s="49"/>
+    </row>
+    <row r="24" spans="1:5" ht="30" customHeight="1">
+      <c r="A24" s="15"/>
+      <c r="B24" s="16"/>
+      <c r="C24" s="47"/>
+      <c r="D24" s="48"/>
+      <c r="E24" s="49"/>
+    </row>
+    <row r="25" spans="1:5" ht="14.25" customHeight="1">
+      <c r="A25" s="15"/>
+      <c r="B25" s="16"/>
+      <c r="C25" s="47"/>
+      <c r="D25" s="48"/>
+      <c r="E25" s="49"/>
+    </row>
+    <row r="26" spans="1:5" ht="14.25" customHeight="1">
+      <c r="A26" s="15"/>
+      <c r="B26" s="16"/>
+      <c r="C26" s="47"/>
+      <c r="D26" s="48"/>
+      <c r="E26" s="49"/>
+    </row>
+    <row r="27" spans="1:5" ht="14.25" customHeight="1">
+      <c r="A27" s="14"/>
+      <c r="B27" s="12"/>
+      <c r="C27" s="50"/>
+      <c r="D27" s="51"/>
+      <c r="E27" s="52"/>
+    </row>
+    <row r="28" spans="1:5" ht="14.25" customHeight="1">
+      <c r="A28" s="13" t="d">
+        <v>2027-03-22</v>
+      </c>
+      <c r="B28" s="11" t="d">
+        <v>2027-04-09</v>
+      </c>
+      <c r="C28" s="23" t="s">
         <v>35</v>
       </c>
-      <c r="D19" s="14"/>
-      <c r="E19" s="37"/>
-    </row>
-    <row r="20" spans="1:5" ht="14.25">
-      <c r="A20" s="6" t="d">
-        <v>2027-01-18</v>
-      </c>
-      <c r="B20" s="51" t="d">
-        <v>2027-03-21</v>
-      </c>
-      <c r="C20" s="38" t="s">
+      <c r="D28" s="24"/>
+      <c r="E28" s="25"/>
+    </row>
+    <row r="29" spans="1:5" ht="14.25" customHeight="1">
+      <c r="A29" s="15"/>
+      <c r="B29" s="16"/>
+      <c r="C29" s="26"/>
+      <c r="D29" s="27"/>
+      <c r="E29" s="28"/>
+    </row>
+    <row r="30" spans="1:5" ht="14.25" customHeight="1">
+      <c r="A30" s="14"/>
+      <c r="B30" s="12"/>
+      <c r="C30" s="29"/>
+      <c r="D30" s="30"/>
+      <c r="E30" s="31"/>
+    </row>
+    <row r="31" spans="1:5" ht="27" customHeight="1">
+      <c r="A31" s="13" t="d">
+        <v>2027-04-12</v>
+      </c>
+      <c r="B31" s="11" t="d">
+        <v>2027-04-23</v>
+      </c>
+      <c r="C31" s="44" t="s">
+        <v>34</v>
+      </c>
+      <c r="D31" s="45"/>
+      <c r="E31" s="46"/>
+    </row>
+    <row r="32" spans="1:5" ht="24" customHeight="1">
+      <c r="A32" s="14"/>
+      <c r="B32" s="12"/>
+      <c r="C32" s="50"/>
+      <c r="D32" s="51"/>
+      <c r="E32" s="52"/>
+    </row>
+    <row r="33" spans="1:5" ht="14.25">
+      <c r="A33" s="13" t="d">
+        <v>2027-04-26</v>
+      </c>
+      <c r="B33" s="11" t="d">
+        <v>2027-06-04</v>
+      </c>
+      <c r="C33" s="53" t="s">
+        <v>31</v>
+      </c>
+      <c r="D33" s="54"/>
+      <c r="E33" s="55"/>
+    </row>
+    <row r="34" spans="1:5" ht="14.25">
+      <c r="A34" s="15"/>
+      <c r="B34" s="16"/>
+      <c r="C34" s="56"/>
+      <c r="D34" s="57"/>
+      <c r="E34" s="58"/>
+    </row>
+    <row r="35" spans="1:5" ht="14.25">
+      <c r="A35" s="15"/>
+      <c r="B35" s="16"/>
+      <c r="C35" s="56"/>
+      <c r="D35" s="57"/>
+      <c r="E35" s="58"/>
+    </row>
+    <row r="36" spans="1:5" ht="14.25">
+      <c r="A36" s="15"/>
+      <c r="B36" s="16"/>
+      <c r="C36" s="56"/>
+      <c r="D36" s="57"/>
+      <c r="E36" s="58"/>
+    </row>
+    <row r="37" spans="1:5" ht="14.25">
+      <c r="A37" s="15"/>
+      <c r="B37" s="16"/>
+      <c r="C37" s="56"/>
+      <c r="D37" s="57"/>
+      <c r="E37" s="58"/>
+    </row>
+    <row r="38" spans="1:5" ht="14.25">
+      <c r="A38" s="14"/>
+      <c r="B38" s="12"/>
+      <c r="C38" s="20"/>
+      <c r="D38" s="21"/>
+      <c r="E38" s="22"/>
+    </row>
+    <row r="39" spans="1:5" ht="14.25">
+      <c r="A39" s="3" t="d">
+        <v>2027-06-07</v>
+      </c>
+      <c r="B39" s="9" t="d">
+        <v>2027-06-11</v>
+      </c>
+      <c r="C39" s="35" t="s">
         <v>36</v>
       </c>
-      <c r="D20" s="15"/>
-      <c r="E20" s="39"/>
-    </row>
-    <row r="21" spans="1:5" ht="14.25" customHeight="1">
-      <c r="A21" s="7"/>
-      <c r="B21" s="53"/>
-      <c r="C21" s="40"/>
-      <c r="D21" s="16"/>
-      <c r="E21" s="41"/>
-    </row>
-    <row r="22" spans="1:5" ht="14.25" customHeight="1">
-      <c r="A22" s="7"/>
-      <c r="B22" s="53"/>
-      <c r="C22" s="40"/>
-      <c r="D22" s="16"/>
-      <c r="E22" s="41"/>
-    </row>
-    <row r="23" spans="1:5" ht="14.25" customHeight="1">
-      <c r="A23" s="7"/>
-      <c r="B23" s="53"/>
-      <c r="C23" s="40"/>
-      <c r="D23" s="16"/>
-      <c r="E23" s="41"/>
-    </row>
-    <row r="24" spans="1:5" ht="14.25" customHeight="1">
-      <c r="A24" s="7"/>
-      <c r="B24" s="53"/>
-      <c r="C24" s="40"/>
-      <c r="D24" s="16"/>
-      <c r="E24" s="41"/>
-    </row>
-    <row r="25" spans="1:5" ht="30" customHeight="1">
-      <c r="A25" s="7"/>
-      <c r="B25" s="53"/>
-      <c r="C25" s="40"/>
-      <c r="D25" s="16"/>
-      <c r="E25" s="41"/>
-    </row>
-    <row r="26" spans="1:5" ht="14.25" customHeight="1">
-      <c r="A26" s="7"/>
-      <c r="B26" s="53"/>
-      <c r="C26" s="40"/>
-      <c r="D26" s="16"/>
-      <c r="E26" s="41"/>
-    </row>
-    <row r="27" spans="1:5" ht="14.25" customHeight="1">
-      <c r="A27" s="7"/>
-      <c r="B27" s="53"/>
-      <c r="C27" s="40"/>
-      <c r="D27" s="16"/>
-      <c r="E27" s="41"/>
-    </row>
-    <row r="28" spans="1:5" ht="14.25" customHeight="1">
-      <c r="A28" s="8"/>
-      <c r="B28" s="52"/>
-      <c r="C28" s="42"/>
-      <c r="D28" s="17"/>
-      <c r="E28" s="43"/>
-    </row>
-    <row r="29" spans="1:5" ht="14.25" customHeight="1">
-      <c r="A29" s="6" t="d">
-        <v>2027-03-22</v>
-      </c>
-      <c r="B29" s="51" t="d">
-        <v>2027-04-09</v>
-      </c>
-      <c r="C29" s="30" t="s">
-        <v>37</v>
-      </c>
-      <c r="D29" s="11"/>
-      <c r="E29" s="31"/>
-    </row>
-    <row r="30" spans="1:5" ht="14.25" customHeight="1">
-      <c r="A30" s="7"/>
-      <c r="B30" s="53"/>
-      <c r="C30" s="32"/>
-      <c r="D30" s="12"/>
-      <c r="E30" s="33"/>
-    </row>
-    <row r="31" spans="1:5" ht="14.25" customHeight="1">
-      <c r="A31" s="8"/>
-      <c r="B31" s="52"/>
-      <c r="C31" s="34"/>
-      <c r="D31" s="13"/>
-      <c r="E31" s="35"/>
-    </row>
-    <row r="32" spans="1:5" ht="27" customHeight="1">
-      <c r="A32" s="6" t="d">
-        <v>2027-04-12</v>
-      </c>
-      <c r="B32" s="51" t="d">
-        <v>2027-04-23</v>
-      </c>
-      <c r="C32" s="38" t="s">
-        <v>36</v>
-      </c>
-      <c r="D32" s="15"/>
-      <c r="E32" s="39"/>
-    </row>
-    <row r="33" spans="1:5" ht="24" customHeight="1">
-      <c r="A33" s="8"/>
-      <c r="B33" s="52"/>
-      <c r="C33" s="42"/>
-      <c r="D33" s="17"/>
-      <c r="E33" s="43"/>
-    </row>
-    <row r="34" spans="1:5" ht="14.25">
-      <c r="A34" s="6" t="d">
-        <v>2027-04-26</v>
-      </c>
-      <c r="B34" s="51" t="d">
-        <v>2027-06-04</v>
-      </c>
-      <c r="C34" s="44" t="s">
-        <v>33</v>
-      </c>
-      <c r="D34" s="9"/>
-      <c r="E34" s="45"/>
-    </row>
-    <row r="35" spans="1:5" ht="14.25">
-      <c r="A35" s="7"/>
-      <c r="B35" s="53"/>
-      <c r="C35" s="46"/>
-      <c r="D35" s="18"/>
-      <c r="E35" s="47"/>
-    </row>
-    <row r="36" spans="1:5" ht="14.25">
-      <c r="A36" s="7"/>
-      <c r="B36" s="53"/>
-      <c r="C36" s="46"/>
-      <c r="D36" s="18"/>
-      <c r="E36" s="47"/>
-    </row>
-    <row r="37" spans="1:5" ht="14.25">
-      <c r="A37" s="7"/>
-      <c r="B37" s="53"/>
-      <c r="C37" s="46"/>
-      <c r="D37" s="18"/>
-      <c r="E37" s="47"/>
-    </row>
-    <row r="38" spans="1:5" ht="14.25">
-      <c r="A38" s="7"/>
-      <c r="B38" s="53"/>
-      <c r="C38" s="46"/>
-      <c r="D38" s="18"/>
-      <c r="E38" s="47"/>
-    </row>
-    <row r="39" spans="1:5" ht="14.25">
-      <c r="A39" s="8"/>
-      <c r="B39" s="52"/>
-      <c r="C39" s="28"/>
-      <c r="D39" s="10"/>
-      <c r="E39" s="29"/>
-    </row>
-    <row r="40" spans="1:5" ht="14.25">
-      <c r="A40" s="3" t="d">
-        <v>2027-06-07</v>
-      </c>
-      <c r="B40" s="54" t="d">
-        <v>2027-06-11</v>
-      </c>
-      <c r="C40" s="48" t="s">
-        <v>38</v>
-      </c>
-      <c r="D40" s="49"/>
-      <c r="E40" s="50"/>
-    </row>
+      <c r="D39" s="36"/>
+      <c r="E39" s="37"/>
+    </row>
+    <row r="40" spans="1:5" ht="14.25" customHeight="1"/>
     <row r="41" spans="1:5" ht="14.25" customHeight="1"/>
     <row r="42" spans="1:5" ht="14.25" customHeight="1"/>
     <row r="43" spans="1:5" ht="14.25" customHeight="1"/>
@@ -2976,34 +2938,33 @@
     <row r="933" ht="14.25" customHeight="1"/>
     <row r="934" ht="14.25" customHeight="1"/>
     <row r="935" ht="14.25" customHeight="1"/>
-    <row r="936" ht="14.25" customHeight="1"/>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="C40:E40"/>
-    <mergeCell ref="E10:E11"/>
-    <mergeCell ref="E12:E13"/>
-    <mergeCell ref="C8:E8"/>
-    <mergeCell ref="E2:E4"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="A14:A15"/>
-    <mergeCell ref="C14:E15"/>
-    <mergeCell ref="C16:E18"/>
-    <mergeCell ref="C19:E19"/>
-    <mergeCell ref="C20:E28"/>
-    <mergeCell ref="B32:B33"/>
-    <mergeCell ref="A32:A33"/>
-    <mergeCell ref="A34:A39"/>
-    <mergeCell ref="B34:B39"/>
-    <mergeCell ref="A16:A18"/>
-    <mergeCell ref="B16:B18"/>
-    <mergeCell ref="C29:E31"/>
-    <mergeCell ref="C32:E33"/>
-    <mergeCell ref="C34:E39"/>
-    <mergeCell ref="B20:B28"/>
-    <mergeCell ref="A20:A28"/>
-    <mergeCell ref="A29:A31"/>
-    <mergeCell ref="B29:B31"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="C39:E39"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="C7:E7"/>
+    <mergeCell ref="E4:E5"/>
+    <mergeCell ref="C19:E27"/>
+    <mergeCell ref="C28:E30"/>
+    <mergeCell ref="C31:E32"/>
+    <mergeCell ref="C33:E38"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="C13:E14"/>
+    <mergeCell ref="C15:E17"/>
+    <mergeCell ref="C18:E18"/>
+    <mergeCell ref="B31:B32"/>
+    <mergeCell ref="A31:A32"/>
+    <mergeCell ref="A33:A38"/>
+    <mergeCell ref="B33:B38"/>
+    <mergeCell ref="A15:A17"/>
+    <mergeCell ref="B15:B17"/>
+    <mergeCell ref="B19:B27"/>
+    <mergeCell ref="A19:A27"/>
+    <mergeCell ref="A28:A30"/>
+    <mergeCell ref="B28:B30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup paperSize="0" fitToWidth="0" fitToHeight="0" orientation="portrait" horizontalDpi="0" verticalDpi="0" copies="0"/>

</xml_diff>

<commit_message>
docs(schedule): update module schedule workbook
</commit_message>
<xml_diff>
--- a/module_schedule.xlsx
+++ b/module_schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://portdotacdotuk-my.sharepoint.com/personal/mani_ghahremani_port_ac_uk/Documents/_Docs/Work Docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E5038DCD-2C1E-4B4A-9BD1-504799618AFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{59FAFAB8-1926-45DD-9FB7-C52E487D5DB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="18960" xr2:uid="{268B58E5-37B1-4943-A657-E8A6B83DFA17}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="40" uniqueCount="37">
+<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="42" uniqueCount="39">
   <si>
     <t>Week beginning Monday</t>
   </si>
@@ -141,7 +141,7 @@
     <t>Lecture 10</t>
   </si>
   <si>
-    <t>Referral Deferral Assessments</t>
+    <t>Exam period</t>
   </si>
   <si>
     <t>Xmas Break</t>
@@ -153,7 +153,13 @@
     <t>Term 2</t>
   </si>
   <si>
+    <t>Referral and Deferral Assessments (for Term 1)</t>
+  </si>
+  <si>
     <t>Easter Break</t>
+  </si>
+  <si>
+    <t>Referral Deferral Assessments (for Term 2)</t>
   </si>
   <si>
     <t>Board week</t>
@@ -255,7 +261,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="36">
+  <borders count="42">
     <border>
       <start/>
       <end/>
@@ -684,6 +690,74 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <start style="medium">
+        <color rgb="FF000000"/>
+      </start>
+      <end/>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <start/>
+      <end style="medium">
+        <color rgb="FF000000"/>
+      </end>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <start/>
+      <end/>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <start style="medium">
+        <color rgb="FF000000"/>
+      </start>
+      <end/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <start/>
+      <end/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <start/>
+      <end style="thin">
+        <color rgb="FF000000"/>
+      </end>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -692,7 +766,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -722,6 +796,108 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="14" fontId="4" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -734,136 +910,58 @@
     <xf numFmtId="14" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="14" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="4" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -892,13 +990,13 @@
   <xdr:twoCellAnchor editAs="absolute">
     <xdr:from>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>561975</xdr:colOff>
+      <xdr:colOff>323850</xdr:colOff>
       <xdr:row>105</xdr:row>
       <xdr:rowOff>79375</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>130175</xdr:colOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>768350</xdr:colOff>
       <xdr:row>113</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
@@ -990,13 +1088,13 @@
   <xdr:twoCellAnchor editAs="absolute">
     <xdr:from>
       <xdr:col>21</xdr:col>
-      <xdr:colOff>1219200</xdr:colOff>
+      <xdr:colOff>981075</xdr:colOff>
       <xdr:row>105</xdr:row>
       <xdr:rowOff>79375</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>22</xdr:col>
-      <xdr:colOff>1254125</xdr:colOff>
+      <xdr:colOff>1016000</xdr:colOff>
       <xdr:row>113</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
@@ -1088,13 +1186,13 @@
   <xdr:twoCellAnchor editAs="absolute">
     <xdr:from>
       <xdr:col>29</xdr:col>
-      <xdr:colOff>276225</xdr:colOff>
+      <xdr:colOff>38100</xdr:colOff>
       <xdr:row>105</xdr:row>
       <xdr:rowOff>79375</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>30</xdr:col>
-      <xdr:colOff>311150</xdr:colOff>
+      <xdr:colOff>73025</xdr:colOff>
       <xdr:row>113</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
@@ -1186,13 +1284,13 @@
   <xdr:twoCellAnchor editAs="absolute">
     <xdr:from>
       <xdr:col>31</xdr:col>
-      <xdr:colOff>819150</xdr:colOff>
+      <xdr:colOff>581025</xdr:colOff>
       <xdr:row>105</xdr:row>
       <xdr:rowOff>79375</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>32</xdr:col>
-      <xdr:colOff>854075</xdr:colOff>
+      <xdr:colOff>615950</xdr:colOff>
       <xdr:row>113</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
@@ -1607,7 +1705,8 @@
   <dimension ref="A1:E935"/>
   <sheetFormatPr defaultColWidth="16.875" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="4" width="17.625" customWidth="1"/>
+    <col min="1" max="1" width="20.75" customWidth="1"/>
+    <col min="2" max="4" width="17.625" customWidth="1"/>
     <col min="5" max="5" width="17.625" style="8" customWidth="1"/>
     <col min="6" max="20" width="11.5" customWidth="1"/>
     <col min="21" max="21" width="16.875" customWidth="1"/>
@@ -1643,7 +1742,7 @@
       <c r="D2" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="E2" s="38" t="s">
+      <c r="E2" s="11" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1660,7 +1759,7 @@
       <c r="D3" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="39"/>
+      <c r="E3" s="12"/>
     </row>
     <row r="4" spans="1:5" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="d">
@@ -1675,7 +1774,7 @@
       <c r="D4" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E4" s="38" t="s">
+      <c r="E4" s="11" t="s">
         <v>12</v>
       </c>
     </row>
@@ -1692,7 +1791,7 @@
       <c r="D5" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="E5" s="39"/>
+      <c r="E5" s="12"/>
     </row>
     <row r="6" spans="1:5" ht="14.25" customHeight="1">
       <c r="A6" s="3" t="d">
@@ -1718,11 +1817,11 @@
       <c r="B7" s="4" t="d">
         <v>2026-10-30</v>
       </c>
-      <c r="C7" s="41" t="s">
+      <c r="C7" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="D7" s="42"/>
-      <c r="E7" s="43"/>
+      <c r="D7" s="18"/>
+      <c r="E7" s="19"/>
     </row>
     <row r="8" spans="1:5" ht="15" customHeight="1">
       <c r="A8" s="3" t="d">
@@ -1754,7 +1853,7 @@
       <c r="D9" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="E9" s="38" t="s">
+      <c r="E9" s="11" t="s">
         <v>23</v>
       </c>
     </row>
@@ -1771,7 +1870,7 @@
       <c r="D10" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="E10" s="39"/>
+      <c r="E10" s="12"/>
     </row>
     <row r="11" spans="1:5" ht="14.25" customHeight="1">
       <c r="A11" s="3" t="d">
@@ -1786,7 +1885,7 @@
       <c r="D11" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="E11" s="38" t="s">
+      <c r="E11" s="11" t="s">
         <v>28</v>
       </c>
     </row>
@@ -1803,54 +1902,54 @@
       <c r="D12" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="E12" s="40"/>
+      <c r="E12" s="16"/>
     </row>
     <row r="13" spans="1:5" ht="14.25">
-      <c r="A13" s="13" t="d">
+      <c r="A13" s="47" t="d">
         <v>2026-12-07</v>
       </c>
-      <c r="B13" s="11" t="d">
+      <c r="B13" s="45" t="d">
         <v>2026-12-18</v>
       </c>
-      <c r="C13" s="17" t="s">
+      <c r="C13" s="49" t="s">
         <v>31</v>
       </c>
-      <c r="D13" s="18"/>
-      <c r="E13" s="19"/>
+      <c r="D13" s="50"/>
+      <c r="E13" s="51"/>
     </row>
     <row r="14" spans="1:5" ht="14.25">
-      <c r="A14" s="14"/>
-      <c r="B14" s="12"/>
-      <c r="C14" s="20"/>
-      <c r="D14" s="21"/>
-      <c r="E14" s="22"/>
+      <c r="A14" s="48"/>
+      <c r="B14" s="46"/>
+      <c r="C14" s="42"/>
+      <c r="D14" s="43"/>
+      <c r="E14" s="44"/>
     </row>
     <row r="15" spans="1:5" ht="14.25" customHeight="1">
-      <c r="A15" s="13" t="d">
+      <c r="A15" s="47" t="d">
         <v>2026-12-21</v>
       </c>
-      <c r="B15" s="11" t="d">
+      <c r="B15" s="45" t="d">
         <v>2026-01-08</v>
       </c>
-      <c r="C15" s="23" t="s">
+      <c r="C15" s="27" t="s">
         <v>32</v>
       </c>
-      <c r="D15" s="24"/>
-      <c r="E15" s="25"/>
+      <c r="D15" s="28"/>
+      <c r="E15" s="29"/>
     </row>
     <row r="16" spans="1:5" ht="14.25" customHeight="1">
-      <c r="A16" s="15"/>
-      <c r="B16" s="16"/>
-      <c r="C16" s="26"/>
-      <c r="D16" s="27"/>
-      <c r="E16" s="28"/>
+      <c r="A16" s="55"/>
+      <c r="B16" s="56"/>
+      <c r="C16" s="30"/>
+      <c r="D16" s="31"/>
+      <c r="E16" s="32"/>
     </row>
     <row r="17" spans="1:5" ht="14.25" customHeight="1">
-      <c r="A17" s="14"/>
-      <c r="B17" s="12"/>
-      <c r="C17" s="29"/>
-      <c r="D17" s="30"/>
-      <c r="E17" s="31"/>
+      <c r="A17" s="48"/>
+      <c r="B17" s="46"/>
+      <c r="C17" s="33"/>
+      <c r="D17" s="34"/>
+      <c r="E17" s="35"/>
     </row>
     <row r="18" spans="1:5" ht="14.25">
       <c r="A18" s="3" t="d">
@@ -1859,175 +1958,211 @@
       <c r="B18" s="9" t="d">
         <v>2027-01-15</v>
       </c>
-      <c r="C18" s="32" t="s">
+      <c r="C18" s="52" t="s">
         <v>33</v>
       </c>
-      <c r="D18" s="33"/>
-      <c r="E18" s="34"/>
+      <c r="D18" s="53"/>
+      <c r="E18" s="54"/>
     </row>
     <row r="19" spans="1:5" ht="14.25">
-      <c r="A19" s="13" t="d">
+      <c r="A19" s="3" t="d">
         <v>2027-01-18</v>
       </c>
-      <c r="B19" s="11" t="d">
-        <v>2027-03-21</v>
-      </c>
-      <c r="C19" s="44" t="s">
+      <c r="B19" s="4" t="d">
+        <v>2027-01-22</v>
+      </c>
+      <c r="C19" s="62" t="s">
         <v>34</v>
       </c>
-      <c r="D19" s="45"/>
-      <c r="E19" s="46"/>
+      <c r="D19" s="21"/>
+      <c r="E19" s="22"/>
     </row>
     <row r="20" spans="1:5" ht="14.25" customHeight="1">
-      <c r="A20" s="15"/>
-      <c r="B20" s="16"/>
-      <c r="C20" s="47"/>
-      <c r="D20" s="48"/>
-      <c r="E20" s="49"/>
+      <c r="A20" s="3" t="d">
+        <v>2027-01-25</v>
+      </c>
+      <c r="B20" s="4" t="d">
+        <v>2027-01-29</v>
+      </c>
+      <c r="C20" s="57"/>
+      <c r="D20" s="58"/>
+      <c r="E20" s="23"/>
     </row>
     <row r="21" spans="1:5" ht="14.25" customHeight="1">
-      <c r="A21" s="15"/>
-      <c r="B21" s="16"/>
-      <c r="C21" s="47"/>
-      <c r="D21" s="48"/>
-      <c r="E21" s="49"/>
+      <c r="A21" s="3" t="d">
+        <v>2027-02-01</v>
+      </c>
+      <c r="B21" s="4" t="d">
+        <v>2027-02-05</v>
+      </c>
+      <c r="C21" s="57"/>
+      <c r="D21" s="58"/>
+      <c r="E21" s="23"/>
     </row>
     <row r="22" spans="1:5" ht="14.25" customHeight="1">
-      <c r="A22" s="15"/>
-      <c r="B22" s="16"/>
-      <c r="C22" s="47"/>
-      <c r="D22" s="48"/>
-      <c r="E22" s="49"/>
+      <c r="A22" s="3" t="d">
+        <v>2027-02-08</v>
+      </c>
+      <c r="B22" s="4" t="d">
+        <v>2027-02-12</v>
+      </c>
+      <c r="C22" s="57"/>
+      <c r="D22" s="58"/>
+      <c r="E22" s="23"/>
     </row>
     <row r="23" spans="1:5" ht="14.25" customHeight="1">
-      <c r="A23" s="15"/>
-      <c r="B23" s="16"/>
-      <c r="C23" s="47"/>
-      <c r="D23" s="48"/>
-      <c r="E23" s="49"/>
+      <c r="A23" s="3" t="d">
+        <v>2027-02-15</v>
+      </c>
+      <c r="B23" s="4" t="d">
+        <v>2027-02-19</v>
+      </c>
+      <c r="C23" s="63"/>
+      <c r="D23" s="64"/>
+      <c r="E23" s="65"/>
     </row>
     <row r="24" spans="1:5" ht="30" customHeight="1">
-      <c r="A24" s="15"/>
-      <c r="B24" s="16"/>
-      <c r="C24" s="47"/>
-      <c r="D24" s="48"/>
-      <c r="E24" s="49"/>
+      <c r="A24" s="3" t="d">
+        <v>2027-02-22</v>
+      </c>
+      <c r="B24" s="4" t="d">
+        <v>2027-02-26</v>
+      </c>
+      <c r="C24" s="59" t="s">
+        <v>35</v>
+      </c>
+      <c r="D24" s="61"/>
+      <c r="E24" s="60"/>
     </row>
     <row r="25" spans="1:5" ht="14.25" customHeight="1">
-      <c r="A25" s="15"/>
-      <c r="B25" s="16"/>
-      <c r="C25" s="47"/>
-      <c r="D25" s="48"/>
-      <c r="E25" s="49"/>
+      <c r="A25" s="3" t="d">
+        <v>2027-03-01</v>
+      </c>
+      <c r="B25" s="4" t="d">
+        <v>2027-03-05</v>
+      </c>
+      <c r="C25" s="62" t="s">
+        <v>34</v>
+      </c>
+      <c r="D25" s="21"/>
+      <c r="E25" s="22"/>
     </row>
     <row r="26" spans="1:5" ht="14.25" customHeight="1">
-      <c r="A26" s="15"/>
-      <c r="B26" s="16"/>
-      <c r="C26" s="47"/>
-      <c r="D26" s="48"/>
-      <c r="E26" s="49"/>
+      <c r="A26" s="3" t="d">
+        <v>2027-03-08</v>
+      </c>
+      <c r="B26" s="4" t="d">
+        <v>2027-03-12</v>
+      </c>
+      <c r="C26" s="57"/>
+      <c r="D26" s="58"/>
+      <c r="E26" s="23"/>
     </row>
     <row r="27" spans="1:5" ht="14.25" customHeight="1">
-      <c r="A27" s="14"/>
-      <c r="B27" s="12"/>
-      <c r="C27" s="50"/>
-      <c r="D27" s="51"/>
-      <c r="E27" s="52"/>
+      <c r="A27" s="3" t="d">
+        <v>2027-03-15</v>
+      </c>
+      <c r="B27" s="4" t="d">
+        <v>2027-03-19</v>
+      </c>
+      <c r="C27" s="66"/>
+      <c r="D27" s="25"/>
+      <c r="E27" s="26"/>
     </row>
     <row r="28" spans="1:5" ht="14.25" customHeight="1">
-      <c r="A28" s="13" t="d">
+      <c r="A28" s="47" t="d">
         <v>2027-03-22</v>
       </c>
-      <c r="B28" s="11" t="d">
+      <c r="B28" s="45" t="d">
         <v>2027-04-09</v>
       </c>
-      <c r="C28" s="23" t="s">
-        <v>35</v>
-      </c>
-      <c r="D28" s="24"/>
-      <c r="E28" s="25"/>
+      <c r="C28" s="27" t="s">
+        <v>36</v>
+      </c>
+      <c r="D28" s="28"/>
+      <c r="E28" s="29"/>
     </row>
     <row r="29" spans="1:5" ht="14.25" customHeight="1">
-      <c r="A29" s="15"/>
-      <c r="B29" s="16"/>
-      <c r="C29" s="26"/>
-      <c r="D29" s="27"/>
-      <c r="E29" s="28"/>
+      <c r="A29" s="55"/>
+      <c r="B29" s="56"/>
+      <c r="C29" s="30"/>
+      <c r="D29" s="31"/>
+      <c r="E29" s="32"/>
     </row>
     <row r="30" spans="1:5" ht="14.25" customHeight="1">
-      <c r="A30" s="14"/>
-      <c r="B30" s="12"/>
-      <c r="C30" s="29"/>
-      <c r="D30" s="30"/>
-      <c r="E30" s="31"/>
+      <c r="A30" s="48"/>
+      <c r="B30" s="46"/>
+      <c r="C30" s="33"/>
+      <c r="D30" s="34"/>
+      <c r="E30" s="35"/>
     </row>
     <row r="31" spans="1:5" ht="27" customHeight="1">
-      <c r="A31" s="13" t="d">
+      <c r="A31" s="47" t="d">
         <v>2027-04-12</v>
       </c>
-      <c r="B31" s="11" t="d">
+      <c r="B31" s="45" t="d">
         <v>2027-04-23</v>
       </c>
-      <c r="C31" s="44" t="s">
+      <c r="C31" s="20" t="s">
         <v>34</v>
       </c>
-      <c r="D31" s="45"/>
-      <c r="E31" s="46"/>
+      <c r="D31" s="21"/>
+      <c r="E31" s="22"/>
     </row>
     <row r="32" spans="1:5" ht="24" customHeight="1">
-      <c r="A32" s="14"/>
-      <c r="B32" s="12"/>
-      <c r="C32" s="50"/>
-      <c r="D32" s="51"/>
-      <c r="E32" s="52"/>
+      <c r="A32" s="48"/>
+      <c r="B32" s="46"/>
+      <c r="C32" s="24"/>
+      <c r="D32" s="25"/>
+      <c r="E32" s="26"/>
     </row>
     <row r="33" spans="1:5" ht="14.25">
-      <c r="A33" s="13" t="d">
+      <c r="A33" s="47" t="d">
         <v>2027-04-26</v>
       </c>
-      <c r="B33" s="11" t="d">
+      <c r="B33" s="45" t="d">
         <v>2027-06-04</v>
       </c>
-      <c r="C33" s="53" t="s">
-        <v>31</v>
-      </c>
-      <c r="D33" s="54"/>
-      <c r="E33" s="55"/>
+      <c r="C33" s="36" t="s">
+        <v>37</v>
+      </c>
+      <c r="D33" s="37"/>
+      <c r="E33" s="38"/>
     </row>
     <row r="34" spans="1:5" ht="14.25">
-      <c r="A34" s="15"/>
-      <c r="B34" s="16"/>
-      <c r="C34" s="56"/>
-      <c r="D34" s="57"/>
-      <c r="E34" s="58"/>
+      <c r="A34" s="55"/>
+      <c r="B34" s="56"/>
+      <c r="C34" s="39"/>
+      <c r="D34" s="40"/>
+      <c r="E34" s="41"/>
     </row>
     <row r="35" spans="1:5" ht="14.25">
-      <c r="A35" s="15"/>
-      <c r="B35" s="16"/>
-      <c r="C35" s="56"/>
-      <c r="D35" s="57"/>
-      <c r="E35" s="58"/>
+      <c r="A35" s="55"/>
+      <c r="B35" s="56"/>
+      <c r="C35" s="39"/>
+      <c r="D35" s="40"/>
+      <c r="E35" s="41"/>
     </row>
     <row r="36" spans="1:5" ht="14.25">
-      <c r="A36" s="15"/>
-      <c r="B36" s="16"/>
-      <c r="C36" s="56"/>
-      <c r="D36" s="57"/>
-      <c r="E36" s="58"/>
+      <c r="A36" s="55"/>
+      <c r="B36" s="56"/>
+      <c r="C36" s="39"/>
+      <c r="D36" s="40"/>
+      <c r="E36" s="41"/>
     </row>
     <row r="37" spans="1:5" ht="14.25">
-      <c r="A37" s="15"/>
-      <c r="B37" s="16"/>
-      <c r="C37" s="56"/>
-      <c r="D37" s="57"/>
-      <c r="E37" s="58"/>
+      <c r="A37" s="55"/>
+      <c r="B37" s="56"/>
+      <c r="C37" s="39"/>
+      <c r="D37" s="40"/>
+      <c r="E37" s="41"/>
     </row>
     <row r="38" spans="1:5" ht="14.25">
-      <c r="A38" s="14"/>
-      <c r="B38" s="12"/>
-      <c r="C38" s="20"/>
-      <c r="D38" s="21"/>
-      <c r="E38" s="22"/>
+      <c r="A38" s="48"/>
+      <c r="B38" s="46"/>
+      <c r="C38" s="42"/>
+      <c r="D38" s="43"/>
+      <c r="E38" s="44"/>
     </row>
     <row r="39" spans="1:5" ht="14.25">
       <c r="A39" s="3" t="d">
@@ -2036,11 +2171,11 @@
       <c r="B39" s="9" t="d">
         <v>2027-06-11</v>
       </c>
-      <c r="C39" s="35" t="s">
-        <v>36</v>
-      </c>
-      <c r="D39" s="36"/>
-      <c r="E39" s="37"/>
+      <c r="C39" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="D39" s="14"/>
+      <c r="E39" s="15"/>
     </row>
     <row r="40" spans="1:5" ht="14.25" customHeight="1"/>
     <row r="41" spans="1:5" ht="14.25" customHeight="1"/>
@@ -2940,31 +3075,31 @@
     <row r="935" ht="14.25" customHeight="1"/>
   </sheetData>
   <mergeCells count="25">
+    <mergeCell ref="B31:B32"/>
+    <mergeCell ref="A31:A32"/>
+    <mergeCell ref="A33:A38"/>
+    <mergeCell ref="B33:B38"/>
+    <mergeCell ref="A15:A17"/>
+    <mergeCell ref="B15:B17"/>
+    <mergeCell ref="A28:A30"/>
+    <mergeCell ref="B28:B30"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="C13:E14"/>
+    <mergeCell ref="C15:E17"/>
+    <mergeCell ref="C18:E18"/>
     <mergeCell ref="E2:E3"/>
     <mergeCell ref="C39:E39"/>
     <mergeCell ref="E9:E10"/>
     <mergeCell ref="E11:E12"/>
     <mergeCell ref="C7:E7"/>
     <mergeCell ref="E4:E5"/>
-    <mergeCell ref="C19:E27"/>
     <mergeCell ref="C28:E30"/>
     <mergeCell ref="C31:E32"/>
     <mergeCell ref="C33:E38"/>
-    <mergeCell ref="B13:B14"/>
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="C13:E14"/>
-    <mergeCell ref="C15:E17"/>
-    <mergeCell ref="C18:E18"/>
-    <mergeCell ref="B31:B32"/>
-    <mergeCell ref="A31:A32"/>
-    <mergeCell ref="A33:A38"/>
-    <mergeCell ref="B33:B38"/>
-    <mergeCell ref="A15:A17"/>
-    <mergeCell ref="B15:B17"/>
-    <mergeCell ref="B19:B27"/>
-    <mergeCell ref="A19:A27"/>
-    <mergeCell ref="A28:A30"/>
-    <mergeCell ref="B28:B30"/>
+    <mergeCell ref="C24:E24"/>
+    <mergeCell ref="C19:E23"/>
+    <mergeCell ref="C25:E27"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup paperSize="0" fitToWidth="0" fitToHeight="0" orientation="portrait" horizontalDpi="0" verticalDpi="0" copies="0"/>

</xml_diff>